<commit_message>
Taking a picture now clears the subwell variables. They can be restored with a butto if desired.
</commit_message>
<xml_diff>
--- a/Resources/Crystal_Sendoff_Sheet.xlsx
+++ b/Resources/Crystal_Sendoff_Sheet.xlsx
@@ -440,7 +440,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K300"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.140625" customWidth="1" min="1" max="1"/>
     <col width="55.28515625" customWidth="1" min="2" max="2"/>
@@ -552,43 +552,14 @@
       <c r="A3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>2TEL_10xHis-2TEL-FIKK2-aggregate_Index__IN_A1_top_left_04-09-2025_07-24-2025-11-31-40_harvested</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>1. (A1) 0.1 M Citric acid pH 3.5, 2.0 M Ammonium sulfate</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>q</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>63</v>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>MJB</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>04-09-2025, 07-24-2025-11-31-40</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None, just a test
-</t>
-        </is>
-      </c>
+      <c r="B3" s="4" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
     </row>
@@ -618,7 +589,7 @@
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
     </row>
@@ -5374,9 +5345,6 @@
       <c r="K300" s="4" t="n"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Made tray variables easier to track. Also improved the chance that running several functions in one session causes no crashes.
</commit_message>
<xml_diff>
--- a/Resources/Crystal_Sendoff_Sheet.xlsx
+++ b/Resources/Crystal_Sendoff_Sheet.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="135" windowWidth="21075" windowHeight="9780" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Crystal_Sendoff_Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191028" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -440,7 +440,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K300"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15.140625" customWidth="1" min="1" max="1"/>
     <col width="55.28515625" customWidth="1" min="2" max="2"/>
@@ -513,37 +513,13 @@
       <c r="A2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_10xHis-1TEL-SR-DARPin_Salt_Rx__SR_E9_bottom_left_05-10-2025_07-12-2025-09-46-20_harvested</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>57. (E9) 1.8 M Sodium phosphate monobasic monohydrate, Potassium phosphate dibasic / pH 6.9</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Long prisms</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>205</v>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Miles Bradford</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>05-10-2025, 07-12-2025-09-46-20</t>
-        </is>
-      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
       <c r="I2" s="4" t="n"/>
       <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="n"/>
@@ -3342,29 +3318,13 @@
       <c r="A189" s="1" t="n">
         <v>189</v>
       </c>
-      <c r="B189" s="4" t="inlineStr">
-        <is>
-          <t>2TEL_10xHis-2TEL-FIKK2-aggregate_Index__IN_H9_bottom_left_04-09-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C189" s="4" t="inlineStr">
-        <is>
-          <t>93. (H9) 0.05 M Zinc acetate dihydrate, 20% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
+      <c r="B189" s="4" t="n"/>
+      <c r="C189" s="4" t="n"/>
       <c r="D189" s="4" t="n"/>
-      <c r="E189" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="F189" s="4" t="n">
-        <v>34</v>
-      </c>
+      <c r="E189" s="4" t="n"/>
+      <c r="F189" s="4" t="n"/>
       <c r="G189" s="4" t="n"/>
-      <c r="H189" s="4" t="inlineStr">
-        <is>
-          <t>04-09-2025, 07-10-2025</t>
-        </is>
-      </c>
+      <c r="H189" s="4" t="n"/>
       <c r="I189" s="4" t="n"/>
       <c r="J189" s="4" t="n"/>
       <c r="K189" s="4" t="n"/>
@@ -3373,33 +3333,13 @@
       <c r="A190" s="1" t="n">
         <v>190</v>
       </c>
-      <c r="B190" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_B4_bottom_left_02-22-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C190" s="4" t="inlineStr">
-        <is>
-          <t>16. (B4) 0.1 M TRIS pH 8.5, 0.3 M Magnesium formate dihydrate</t>
-        </is>
-      </c>
+      <c r="B190" s="4" t="n"/>
+      <c r="C190" s="4" t="n"/>
       <c r="D190" s="4" t="n"/>
-      <c r="E190" s="4" t="n">
-        <v>89</v>
-      </c>
-      <c r="F190" s="4" t="n">
-        <v>101</v>
-      </c>
-      <c r="G190" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H190" s="4" t="inlineStr">
-        <is>
-          <t>02-22-2025, 07-10-2025</t>
-        </is>
-      </c>
+      <c r="E190" s="4" t="n"/>
+      <c r="F190" s="4" t="n"/>
+      <c r="G190" s="4" t="n"/>
+      <c r="H190" s="4" t="n"/>
       <c r="I190" s="4" t="n"/>
       <c r="J190" s="4" t="n"/>
       <c r="K190" s="4" t="n"/>
@@ -3408,33 +3348,13 @@
       <c r="A191" s="1" t="n">
         <v>191</v>
       </c>
-      <c r="B191" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_B4_bottom_left_02-22-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C191" s="4" t="inlineStr">
-        <is>
-          <t>16. (B4) 0.1 M TRIS pH 8.5, 0.3 M Magnesium formate dihydrate</t>
-        </is>
-      </c>
+      <c r="B191" s="4" t="n"/>
+      <c r="C191" s="4" t="n"/>
       <c r="D191" s="4" t="n"/>
-      <c r="E191" s="4" t="n">
-        <v>89</v>
-      </c>
-      <c r="F191" s="4" t="n">
-        <v>101</v>
-      </c>
-      <c r="G191" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H191" s="4" t="inlineStr">
-        <is>
-          <t>02-22-2025, 07-10-2025</t>
-        </is>
-      </c>
+      <c r="E191" s="4" t="n"/>
+      <c r="F191" s="4" t="n"/>
+      <c r="G191" s="4" t="n"/>
+      <c r="H191" s="4" t="n"/>
       <c r="I191" s="4" t="n"/>
       <c r="J191" s="4" t="n"/>
       <c r="K191" s="4" t="n"/>
@@ -3443,33 +3363,13 @@
       <c r="A192" s="1" t="n">
         <v>192</v>
       </c>
-      <c r="B192" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_B4_bottom_left_02-22-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C192" s="4" t="inlineStr">
-        <is>
-          <t>16. (B4) 0.1 M TRIS pH 8.5, 0.3 M Magnesium formate dihydrate</t>
-        </is>
-      </c>
+      <c r="B192" s="4" t="n"/>
+      <c r="C192" s="4" t="n"/>
       <c r="D192" s="4" t="n"/>
-      <c r="E192" s="4" t="n">
-        <v>89</v>
-      </c>
-      <c r="F192" s="4" t="n">
-        <v>101</v>
-      </c>
-      <c r="G192" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H192" s="4" t="inlineStr">
-        <is>
-          <t>02-22-2025, 07-10-2025</t>
-        </is>
-      </c>
+      <c r="E192" s="4" t="n"/>
+      <c r="F192" s="4" t="n"/>
+      <c r="G192" s="4" t="n"/>
+      <c r="H192" s="4" t="n"/>
       <c r="I192" s="4" t="n"/>
       <c r="J192" s="4" t="n"/>
       <c r="K192" s="4" t="n"/>
@@ -3478,11 +3378,7 @@
       <c r="A193" s="1" t="n">
         <v>193</v>
       </c>
-      <c r="B193" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_F8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
+      <c r="B193" s="4" t="n"/>
       <c r="J193" s="4" t="n"/>
       <c r="K193" s="4" t="n"/>
     </row>
@@ -3490,43 +3386,14 @@
       <c r="A194" s="1" t="n">
         <v>194</v>
       </c>
-      <c r="B194" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C194" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D194" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E194" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F194" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G194" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H194" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I194" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B194" s="4" t="n"/>
+      <c r="C194" s="4" t="n"/>
+      <c r="D194" s="4" t="n"/>
+      <c r="E194" s="4" t="n"/>
+      <c r="F194" s="4" t="n"/>
+      <c r="G194" s="4" t="n"/>
+      <c r="H194" s="4" t="n"/>
+      <c r="I194" s="4" t="n"/>
       <c r="J194" s="4" t="n"/>
       <c r="K194" s="4" t="n"/>
     </row>
@@ -3534,43 +3401,14 @@
       <c r="A195" s="1" t="n">
         <v>195</v>
       </c>
-      <c r="B195" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C195" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D195" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E195" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F195" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G195" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H195" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I195" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B195" s="4" t="n"/>
+      <c r="C195" s="4" t="n"/>
+      <c r="D195" s="4" t="n"/>
+      <c r="E195" s="4" t="n"/>
+      <c r="F195" s="4" t="n"/>
+      <c r="G195" s="4" t="n"/>
+      <c r="H195" s="4" t="n"/>
+      <c r="I195" s="4" t="n"/>
       <c r="J195" s="4" t="n"/>
       <c r="K195" s="4" t="n"/>
     </row>
@@ -3578,43 +3416,14 @@
       <c r="A196" s="1" t="n">
         <v>196</v>
       </c>
-      <c r="B196" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C196" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D196" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E196" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F196" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G196" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H196" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I196" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B196" s="4" t="n"/>
+      <c r="C196" s="4" t="n"/>
+      <c r="D196" s="4" t="n"/>
+      <c r="E196" s="4" t="n"/>
+      <c r="F196" s="4" t="n"/>
+      <c r="G196" s="4" t="n"/>
+      <c r="H196" s="4" t="n"/>
+      <c r="I196" s="4" t="n"/>
       <c r="J196" s="4" t="n"/>
       <c r="K196" s="4" t="n"/>
     </row>
@@ -3622,43 +3431,14 @@
       <c r="A197" s="1" t="n">
         <v>197</v>
       </c>
-      <c r="B197" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C197" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D197" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E197" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F197" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G197" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H197" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I197" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B197" s="4" t="n"/>
+      <c r="C197" s="4" t="n"/>
+      <c r="D197" s="4" t="n"/>
+      <c r="E197" s="4" t="n"/>
+      <c r="F197" s="4" t="n"/>
+      <c r="G197" s="4" t="n"/>
+      <c r="H197" s="4" t="n"/>
+      <c r="I197" s="4" t="n"/>
       <c r="J197" s="4" t="n"/>
       <c r="K197" s="4" t="n"/>
     </row>
@@ -3666,43 +3446,14 @@
       <c r="A198" s="1" t="n">
         <v>198</v>
       </c>
-      <c r="B198" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C198" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D198" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E198" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F198" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G198" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H198" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I198" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B198" s="4" t="n"/>
+      <c r="C198" s="4" t="n"/>
+      <c r="D198" s="4" t="n"/>
+      <c r="E198" s="4" t="n"/>
+      <c r="F198" s="4" t="n"/>
+      <c r="G198" s="4" t="n"/>
+      <c r="H198" s="4" t="n"/>
+      <c r="I198" s="4" t="n"/>
       <c r="J198" s="4" t="n"/>
       <c r="K198" s="4" t="n"/>
     </row>
@@ -3732,43 +3483,14 @@
       <c r="A201" s="1" t="n">
         <v>201</v>
       </c>
-      <c r="B201" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C201" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D201" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E201" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F201" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G201" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H201" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I201" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B201" s="4" t="n"/>
+      <c r="C201" s="4" t="n"/>
+      <c r="D201" s="4" t="n"/>
+      <c r="E201" s="4" t="n"/>
+      <c r="F201" s="4" t="n"/>
+      <c r="G201" s="4" t="n"/>
+      <c r="H201" s="4" t="n"/>
+      <c r="I201" s="4" t="n"/>
       <c r="J201" s="4" t="n"/>
       <c r="K201" s="4" t="n"/>
     </row>
@@ -3776,43 +3498,14 @@
       <c r="A202" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="B202" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C202" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D202" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E202" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F202" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G202" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H202" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I202" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B202" s="4" t="n"/>
+      <c r="C202" s="4" t="n"/>
+      <c r="D202" s="4" t="n"/>
+      <c r="E202" s="4" t="n"/>
+      <c r="F202" s="4" t="n"/>
+      <c r="G202" s="4" t="n"/>
+      <c r="H202" s="4" t="n"/>
+      <c r="I202" s="4" t="n"/>
       <c r="J202" s="4" t="n"/>
       <c r="K202" s="4" t="n"/>
     </row>
@@ -3820,43 +3513,14 @@
       <c r="A203" s="1" t="n">
         <v>203</v>
       </c>
-      <c r="B203" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C203" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D203" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E203" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F203" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G203" s="4" t="inlineStr">
-        <is>
-          <t>Wisdom</t>
-        </is>
-      </c>
-      <c r="H203" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I203" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B203" s="4" t="n"/>
+      <c r="C203" s="4" t="n"/>
+      <c r="D203" s="4" t="n"/>
+      <c r="E203" s="4" t="n"/>
+      <c r="F203" s="4" t="n"/>
+      <c r="G203" s="4" t="n"/>
+      <c r="H203" s="4" t="n"/>
+      <c r="I203" s="4" t="n"/>
       <c r="J203" s="4" t="n"/>
       <c r="K203" s="4" t="n"/>
     </row>
@@ -3864,43 +3528,14 @@
       <c r="A204" s="1" t="n">
         <v>204</v>
       </c>
-      <c r="B204" s="4" t="inlineStr">
-        <is>
-          <t>1TEL_CMG2_Index__IN_H8_bottom_left_05-27-2025_07-10-2025_harvested</t>
-        </is>
-      </c>
-      <c r="C204" s="4" t="inlineStr">
-        <is>
-          <t>92. (H8) 0.1 M Magnesium formate dihydrate, 15% w/v Polyethylene glycol 3,350</t>
-        </is>
-      </c>
-      <c r="D204" s="4" t="inlineStr">
-        <is>
-          <t>Rectangle</t>
-        </is>
-      </c>
-      <c r="E204" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="F204" s="4" t="n">
-        <v>130</v>
-      </c>
-      <c r="G204" s="4" t="inlineStr">
-        <is>
-          <t>Jamison</t>
-        </is>
-      </c>
-      <c r="H204" s="4" t="inlineStr">
-        <is>
-          <t>05-27-2025, 07-10-2025</t>
-        </is>
-      </c>
-      <c r="I204" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Double crystal
-</t>
-        </is>
-      </c>
+      <c r="B204" s="4" t="n"/>
+      <c r="C204" s="4" t="n"/>
+      <c r="D204" s="4" t="n"/>
+      <c r="E204" s="4" t="n"/>
+      <c r="F204" s="4" t="n"/>
+      <c r="G204" s="4" t="n"/>
+      <c r="H204" s="4" t="n"/>
+      <c r="I204" s="4" t="n"/>
       <c r="J204" s="4" t="n"/>
       <c r="K204" s="4" t="n"/>
     </row>

</xml_diff>